<commit_message>
feat: tighten site quality and add application gallery
</commit_message>
<xml_diff>
--- a/docs/MCCS_CF_Product_Specifications.xlsx
+++ b/docs/MCCS_CF_Product_Specifications.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF 产品规格" sheetId="1" r:id="R338186c641ff4d83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购说明" sheetId="2" r:id="R74de7c8ad19a48ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CF 产品规格" sheetId="1" r:id="R5020a3e5a1c443da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购说明" sheetId="2" r:id="Rd5c70789d4fd4e48"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -506,7 +506,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>公开采购规格表 | 29 个 CF 型号 | 尺寸与穴盘适配请在打样前按图纸或实物复核 | Updated 2026-09-01</x:v>
+        <x:v>公开采购规格表 | 28 个 CF 型号 | 尺寸与穴盘适配请在打样前按图纸或实物复核 | Updated 2026-09-01</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -1264,25 +1264,25 @@
     </x:row>
     <x:row r="27" ht="46" customHeight="1">
       <x:c r="A27" s="34" t="str">
-        <x:v>CF-2735</x:v>
+        <x:v>CF-3038</x:v>
       </x:c>
       <x:c r="B27" s="17" t="str">
-        <x:v>紧凑型组培基质块 3.5 cm</x:v>
+        <x:v>扦插育苗块 3.8 cm</x:v>
       </x:c>
       <x:c r="C27" s="17" t="str">
-        <x:v>Tissue Culture Propagation Plug 3.5 cm</x:v>
+        <x:v>Cuttings Propagation Plug 3.8 cm</x:v>
       </x:c>
       <x:c r="D27" s="17" t="str">
-        <x:v>组培基质块 / Tissue Culture Plug</x:v>
+        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="E27" s="17" t="str">
-        <x:v>Top Ø 2.7 cm / Bottom Ø 2.3 cm / Height 3.5 cm</x:v>
+        <x:v>Top Ø 3.0 cm / Bottom Ø 2.2 cm / Height 3.8 cm</x:v>
       </x:c>
       <x:c r="F27" s="17" t="str">
-        <x:v>180-cell propagation tray</x:v>
+        <x:v>Confirm against the buyer's tray drawing or physical sample</x:v>
       </x:c>
       <x:c r="G27" s="17" t="str">
-        <x:v>Tissue-culture acclimatization and compact high-count trays</x:v>
+        <x:v>Commercial cuttings propagation and model-to-tray trials</x:v>
       </x:c>
       <x:c r="H27" s="17" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
@@ -1291,30 +1291,30 @@
         <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J27" s="17" t="str">
-        <x:v>assets/products/CF-2735-factory.webp</x:v>
+        <x:v>assets/products/CF-3038-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="46" customHeight="1">
       <x:c r="A28" s="36" t="str">
-        <x:v>CF-3038</x:v>
+        <x:v>CF-3038B</x:v>
       </x:c>
       <x:c r="B28" s="37" t="str">
-        <x:v>扦插育苗块 3.8 cm</x:v>
+        <x:v>水培育苗块 3.8 cm B 型</x:v>
       </x:c>
       <x:c r="C28" s="37" t="str">
-        <x:v>Cuttings Propagation Plug 3.8 cm</x:v>
+        <x:v>Hydroponic Propagation Plug 3.8 cm</x:v>
       </x:c>
       <x:c r="D28" s="37" t="str">
-        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
+        <x:v>水培育苗块 / Hydroponic Plug</x:v>
       </x:c>
       <x:c r="E28" s="37" t="str">
         <x:v>Top Ø 3.0 cm / Bottom Ø 2.2 cm / Height 3.8 cm</x:v>
       </x:c>
       <x:c r="F28" s="37" t="str">
-        <x:v>Confirm against the buyer's tray drawing or physical sample</x:v>
+        <x:v>Confirm against the buyer's hydroponic tray or holder</x:v>
       </x:c>
       <x:c r="G28" s="37" t="str">
-        <x:v>Commercial cuttings propagation and model-to-tray trials</x:v>
+        <x:v>Hydroponic sowing, nursery production and controlled-environment systems</x:v>
       </x:c>
       <x:c r="H28" s="37" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
@@ -1323,30 +1323,30 @@
         <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J28" s="37" t="str">
-        <x:v>assets/products/CF-3038-factory.webp</x:v>
+        <x:v>assets/products/CF-3038B-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="46" customHeight="1">
       <x:c r="A29" s="34" t="str">
-        <x:v>CF-3038B</x:v>
+        <x:v>CF-3545</x:v>
       </x:c>
       <x:c r="B29" s="17" t="str">
-        <x:v>水培育苗块 3.8 cm B 型</x:v>
+        <x:v>水培育苗块 4.5 cm</x:v>
       </x:c>
       <x:c r="C29" s="17" t="str">
-        <x:v>Hydroponic Propagation Plug 3.8 cm</x:v>
+        <x:v>Hydroponic Propagation Plug 4.5 cm</x:v>
       </x:c>
       <x:c r="D29" s="17" t="str">
         <x:v>水培育苗块 / Hydroponic Plug</x:v>
       </x:c>
       <x:c r="E29" s="17" t="str">
-        <x:v>Top Ø 3.0 cm / Bottom Ø 2.2 cm / Height 3.8 cm</x:v>
+        <x:v>Top Ø 3.5 cm / Bottom Ø 2.2 cm / Height 4.5 cm</x:v>
       </x:c>
       <x:c r="F29" s="17" t="str">
         <x:v>Confirm against the buyer's hydroponic tray or holder</x:v>
       </x:c>
       <x:c r="G29" s="17" t="str">
-        <x:v>Hydroponic sowing, nursery production and controlled-environment systems</x:v>
+        <x:v>Hydroponic propagation and controlled-environment nursery production</x:v>
       </x:c>
       <x:c r="H29" s="17" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
@@ -1355,136 +1355,116 @@
         <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J29" s="17" t="str">
-        <x:v>assets/products/CF-3038B-factory.webp</x:v>
+        <x:v>assets/products/CF-3545-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="46" customHeight="1">
       <x:c r="A30" s="36" t="str">
-        <x:v>CF-3545</x:v>
+        <x:v>CF-3550</x:v>
       </x:c>
       <x:c r="B30" s="37" t="str">
-        <x:v>水培育苗块 4.5 cm</x:v>
+        <x:v>高型育苗块 5.3 cm</x:v>
       </x:c>
       <x:c r="C30" s="37" t="str">
-        <x:v>Hydroponic Propagation Plug 4.5 cm</x:v>
+        <x:v>Tall Nursery Plug 5.3 cm</x:v>
       </x:c>
       <x:c r="D30" s="37" t="str">
-        <x:v>水培育苗块 / Hydroponic Plug</x:v>
+        <x:v>育苗基质块 / Seedling Plug</x:v>
       </x:c>
       <x:c r="E30" s="37" t="str">
-        <x:v>Top Ø 3.5 cm / Bottom Ø 2.2 cm / Height 4.5 cm</x:v>
+        <x:v>Top Ø 3.7 cm / Bottom Ø 2.2 cm / Height 5.3 cm</x:v>
       </x:c>
       <x:c r="F30" s="37" t="str">
-        <x:v>Confirm against the buyer's hydroponic tray or holder</x:v>
+        <x:v>Deeper nursery and propagation trays with approximately 3.7 cm openings</x:v>
       </x:c>
       <x:c r="G30" s="37" t="str">
-        <x:v>Hydroponic propagation and controlled-environment nursery production</x:v>
+        <x:v>Seedlings and cuttings requiring a taller propagation format</x:v>
       </x:c>
       <x:c r="H30" s="37" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
       </x:c>
       <x:c r="I30" s="37" t="str">
-        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
+        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J30" s="37" t="str">
-        <x:v>assets/products/CF-3545-factory.webp</x:v>
+        <x:v>assets/products/CF-3550.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="46" customHeight="1">
       <x:c r="A31" s="34" t="str">
-        <x:v>CF-3550</x:v>
+        <x:v>CF-5050</x:v>
       </x:c>
       <x:c r="B31" s="17" t="str">
-        <x:v>高型育苗块 5.3 cm</x:v>
+        <x:v>50 穴扦插育苗块 5.0 cm</x:v>
       </x:c>
       <x:c r="C31" s="17" t="str">
-        <x:v>Tall Nursery Plug 5.3 cm</x:v>
+        <x:v>50-Cell Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="D31" s="17" t="str">
-        <x:v>育苗基质块 / Seedling Plug</x:v>
+        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
       </x:c>
       <x:c r="E31" s="17" t="str">
-        <x:v>Top Ø 3.7 cm / Bottom Ø 2.2 cm / Height 5.3 cm</x:v>
+        <x:v>Top Ø 5.0 cm / Bottom Ø 3.8 cm / Height 5.0 cm</x:v>
       </x:c>
       <x:c r="F31" s="17" t="str">
-        <x:v>Deeper nursery and propagation trays with approximately 3.7 cm openings</x:v>
+        <x:v>50-cell propagation tray</x:v>
       </x:c>
       <x:c r="G31" s="17" t="str">
-        <x:v>Seedlings and cuttings requiring a taller propagation format</x:v>
+        <x:v>Larger cuttings and commercial 50-cell nursery workflows</x:v>
       </x:c>
       <x:c r="H31" s="17" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
       </x:c>
       <x:c r="I31" s="17" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
+        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
       </x:c>
       <x:c r="J31" s="17" t="str">
-        <x:v>assets/products/CF-3550.webp</x:v>
+        <x:v>assets/products/CF-5050-factory.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="46" customHeight="1">
       <x:c r="A32" s="36" t="str">
-        <x:v>CF-5050</x:v>
+        <x:v>CF-7050</x:v>
       </x:c>
       <x:c r="B32" s="37" t="str">
-        <x:v>50 穴扦插育苗块 5.0 cm</x:v>
+        <x:v>高型育苗块 6.8 cm</x:v>
       </x:c>
       <x:c r="C32" s="37" t="str">
-        <x:v>50-Cell Cuttings Propagation Plug</x:v>
+        <x:v>Tall Nursery Plug 6.8 cm</x:v>
       </x:c>
       <x:c r="D32" s="37" t="str">
-        <x:v>扦插育苗块 / Cuttings Propagation Plug</x:v>
+        <x:v>育苗基质块 / Seedling Plug</x:v>
       </x:c>
       <x:c r="E32" s="37" t="str">
-        <x:v>Top Ø 5.0 cm / Bottom Ø 3.8 cm / Height 5.0 cm</x:v>
+        <x:v>Top Ø 4.8 cm / Bottom Ø 3.5 cm / Height 6.8 cm</x:v>
       </x:c>
       <x:c r="F32" s="37" t="str">
-        <x:v>50-cell propagation tray</x:v>
+        <x:v>Deep nursery trays, pots or holders with approximately 4.8 cm openings</x:v>
       </x:c>
       <x:c r="G32" s="37" t="str">
-        <x:v>Larger cuttings and commercial 50-cell nursery workflows</x:v>
+        <x:v>Larger seedlings, deeper rooting stages and transplant programs</x:v>
       </x:c>
       <x:c r="H32" s="37" t="str">
         <x:v>Confirm after carton size and packaging format are approved.</x:v>
       </x:c>
       <x:c r="I32" s="37" t="str">
-        <x:v>Dimensions and application cross-checked against the factory website.</x:v>
+        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
       </x:c>
       <x:c r="J32" s="37" t="str">
-        <x:v>assets/products/CF-5050-factory.webp</x:v>
+        <x:v>assets/products/CF-7050.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="46" customHeight="1">
-      <x:c r="A33" s="35" t="str">
-        <x:v>CF-7050</x:v>
-      </x:c>
-      <x:c r="B33" s="18" t="str">
-        <x:v>高型育苗块 6.8 cm</x:v>
-      </x:c>
-      <x:c r="C33" s="18" t="str">
-        <x:v>Tall Nursery Plug 6.8 cm</x:v>
-      </x:c>
-      <x:c r="D33" s="18" t="str">
-        <x:v>育苗基质块 / Seedling Plug</x:v>
-      </x:c>
-      <x:c r="E33" s="18" t="str">
-        <x:v>Top Ø 4.8 cm / Bottom Ø 3.5 cm / Height 6.8 cm</x:v>
-      </x:c>
-      <x:c r="F33" s="18" t="str">
-        <x:v>Deep nursery trays, pots or holders with approximately 4.8 cm openings</x:v>
-      </x:c>
-      <x:c r="G33" s="18" t="str">
-        <x:v>Larger seedlings, deeper rooting stages and transplant programs</x:v>
-      </x:c>
-      <x:c r="H33" s="18" t="str">
-        <x:v>Confirm after carton size and packaging format are approved.</x:v>
-      </x:c>
-      <x:c r="I33" s="18" t="str">
-        <x:v>Listed in the approved product catalog; confirm the current production drawing during sampling.</x:v>
-      </x:c>
-      <x:c r="J33" s="18" t="str">
-        <x:v>assets/products/CF-7050.webp</x:v>
-      </x:c>
+      <x:c r="A33"/>
+      <x:c r="B33"/>
+      <x:c r="C33"/>
+      <x:c r="D33"/>
+      <x:c r="E33"/>
+      <x:c r="F33"/>
+      <x:c r="G33"/>
+      <x:c r="H33"/>
+      <x:c r="I33"/>
+      <x:c r="J33"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1493,7 +1473,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98ccd90b0b0c4737"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3ec2c7412ab452b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>